<commit_message>
Update make_seed.py and add generated FAQ seed sheet
</commit_message>
<xml_diff>
--- a/docs/이랜드건설_동료평가_피어피드백.xlsx
+++ b/docs/이랜드건설_동료평가_피어피드백.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="동료평가_피어피드백" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="점수산정_기준" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="동료평가_FAQ_시드" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="동료평가_피어피드백" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="점수산정_기준" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="동료평가_FAQ_시드" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="이랜드건설_동료평가_피어피드백_FAQ_시드" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -118,7 +119,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -140,11 +141,55 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -197,6 +242,8 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -935,6 +982,12 @@
           <t>【운영 방식】 구글폼 → 동료 선택(가나다순) → 지식/태도 각 4문항 응답 → 최소 3명 평가 → 제출 | 데이터 수집 후 HR팀이 엑셀 다운로드하여 수동 분석 (자동화 필요 영역)</t>
         </is>
       </c>
+      <c r="B12" s="18" t="n"/>
+      <c r="C12" s="18" t="n"/>
+      <c r="D12" s="18" t="n"/>
+      <c r="E12" s="18" t="n"/>
+      <c r="F12" s="18" t="n"/>
+      <c r="G12" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1123,12 +1176,17 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
           <t>총점 = (긍정 4문항 합산) + (개선 4문항 역산 합산) → 만점 40점 → 100점 환산: 총점/40×100</t>
         </is>
       </c>
+      <c r="B9" s="18" t="n"/>
+      <c r="C9" s="18" t="n"/>
+      <c r="D9" s="18" t="n"/>
+      <c r="E9" s="19" t="n"/>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="15" t="inlineStr">
@@ -1136,6 +1194,10 @@
           <t>승진 연계 기준: 대리 승진 시 70점 이상 / 과장 승진 시 75점 이상 / 차장 승진 시 80점 이상 (승진기준_종합 시트 연계)</t>
         </is>
       </c>
+      <c r="B10" s="18" t="n"/>
+      <c r="C10" s="18" t="n"/>
+      <c r="D10" s="18" t="n"/>
+      <c r="E10" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1307,4 +1369,229 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>이랜드건설_동료평가_피어피드백 FAQ 시드 (자동 생성)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>카테고리</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>질문</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>답변</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>평가/승진</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>동료평가(피어피드백)는 연간 몇 회 실시되나요?</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>연 2회 실시합니다. 상반기와 하반기에 각각 1회씩 진행됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>평가/승진</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>동료평가에서 최소 몇 명 이상의 평가를 받아야 하나요?</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>최소 3명 이상의 동료로부터 평가를 받아야 합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>평가/승진</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>피어피드백 평가 항목은 어떻게 구성되어 있나요?</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>지식(Knowledge) 영역 4문항과 태도(Attitude) 영역 4문항, 총 8문항으로 구성됩니다. 지식은 직무 전문성, 직무 역량, 성장 필요, 배치 적합성을 평가하고, 태도는 멘토십, 협업·배려, 조직 문화, 대인관계를 평가합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>평가/승진</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>동료평가 최종 점수는 어떻게 산정되나요?</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>긍정 문항 4개와 개선(역방향) 문항 4개를 합산하여 만점 40점을 기준으로 합니다. 개선 문항은 역산되어 계산됩니다. 최종적으로 총점을 40으로 나누고 100을 곱하여 100점 만점으로 환산됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>평가/승진</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>대리로 승진하려면 동료평가에서 몇 점 이상을 받아야 하나요?</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>대리 승진 시 피어피드백 70점 이상이 필요합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>평가/승진</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>과장으로 승진하려면 동료평가에서 몇 점 이상을 받아야 하나요?</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>과장 승진 시 피어피드백 75점 이상이 필요합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>평가/승진</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>차장으로 승진하려면 동료평가에서 몇 점 이상을 받아야 하나요?</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>차장 승진 시 피어피드백 80점 이상이 필요합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>평가/승진</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>개선 문항에서 "매우 그렇다"고 평가받으면 몇 점이 되나요?</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>개선 문항에서 "매우 그렇다"(5점)로 평가받으면 역산되어 1점이 됩니다. 이는 개선이 필요 없다는 의미로 해석됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>평가/승진</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>긍정 문항과 개선 문항의 점수 차이는 무엇인가요?</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>긍정 문항은 응답 그대로 점수가 적용되고, 개선 문항은 역산됩니다. 예를 들어 개선 문항에서 "그렇지 않다"(2점)고 평가받으면 역산되어 4점이 됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>평가/승진</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>동료평가는 어떤 시스템으로 운영되나요?</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>구글폼 기반으로 운영됩니다. 동료를 선택한 후 지식과 태도 각 4문항에 응답하는 방식입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>평가/승진</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>동료평가 문항 중 "이랜드 스피릿을 더 학습하고 실천하면 좋겠습니다"는 어떤 항목인가요?</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>이는 태도 영역의 조직 문화 항목으로, 개선 문항입니다. 조직 문화 적합도를 평가하는 문항이며 역산되어 계산됩니다.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs 업데이트 (2026-05-29 00:50)
</commit_message>
<xml_diff>
--- a/docs/이랜드건설_동료평가_피어피드백.xlsx
+++ b/docs/이랜드건설_동료평가_피어피드백.xlsx
@@ -1377,7 +1377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1412,12 +1412,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>동료평가(피어피드백)는 연간 몇 회 실시되나요?</t>
+          <t>동료평가(피어피드백)는 몇 년에 몇 번 실시되나요?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>연 2회 실시합니다. 상반기와 하반기에 각각 1회씩 진행됩니다.</t>
+          <t>연 2회(상반기, 하반기)에 걸쳐 실시됩니다.</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>동료평가에서 최소 몇 명 이상의 평가를 받아야 하나요?</t>
+          <t>동료평가에서 최소 몇 명의 평가를 받아야 하나요?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1446,12 +1446,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>피어피드백 평가 항목은 어떻게 구성되어 있나요?</t>
+          <t>동료평가 점수는 어떻게 계산되나요?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>지식(Knowledge) 영역 4문항과 태도(Attitude) 영역 4문항, 총 8문항으로 구성됩니다. 지식은 직무 전문성, 직무 역량, 성장 필요, 배치 적합성을 평가하고, 태도는 멘토십, 협업·배려, 조직 문화, 대인관계를 평가합니다.</t>
+          <t>지식 4문항과 태도 4문항으로 총 8문항을 5점 척도로 평가합니다. 긍정 문항은 그대로 계산하고, 개선 문항(지식3·4, 태도3·4)은 역산하여 합산한 후 40점 만점을 100점으로 환산합니다.</t>
         </is>
       </c>
     </row>
@@ -1463,12 +1463,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>동료평가 최종 점수는 어떻게 산정되나요?</t>
+          <t>동료평가에서 "개선 문항"이란 무엇인가요?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>긍정 문항 4개와 개선(역방향) 문항 4개를 합산하여 만점 40점을 기준으로 합니다. 개선 문항은 역산되어 계산됩니다. 최종적으로 총점을 40으로 나누고 100을 곱하여 100점 만점으로 환산됩니다.</t>
+          <t>개선 문항은 역방향 문항으로, 응답 점수를 역산하여 계산합니다. 지식 3·4번(성장 필요, 배치 적합성)과 태도 3·4번(조직 문화, 대인관계) 4개 문항이 해당됩니다. 예를 들어 "매우 그렇다"에 응답하면 1점으로 역산됩니다.</t>
         </is>
       </c>
     </row>
@@ -1480,12 +1480,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>대리로 승진하려면 동료평가에서 몇 점 이상을 받아야 하나요?</t>
+          <t>대리로 승진하려면 동료평가 점수가 몇 점 이상이어야 하나요?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>대리 승진 시 피어피드백 70점 이상이 필요합니다.</t>
+          <t>대리 승진 시 70점 이상, 과장 승진 시 75점 이상, 차장 승진 시 80점 이상이어야 합니다.</t>
         </is>
       </c>
     </row>
@@ -1497,12 +1497,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>과장으로 승진하려면 동료평가에서 몇 점 이상을 받아야 하나요?</t>
+          <t>동료평가의 지식 영역에서는 어떤 항목들을 평가하나요?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>과장 승진 시 피어피드백 75점 이상이 필요합니다.</t>
+          <t>직무 전문성(사내 강사 추천 여부), 직무 역량(연차 대비 역량 수준), 성장 필요도, 배치 적합성 등 4개 항목을 평가합니다.</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>차장으로 승진하려면 동료평가에서 몇 점 이상을 받아야 하나요?</t>
+          <t>동료평가의 태도 영역에서는 어떤 항목들을 평가하나요?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>차장 승진 시 피어피드백 80점 이상이 필요합니다.</t>
+          <t>멘토십(인격적 멘토 역할), 협업·배려(동료 배려 및 존중), 조직 문화(이랜드 스피릿 실천), 대인관계(관계 개선 필요도) 등 4개 항목을 평가합니다.</t>
         </is>
       </c>
     </row>
@@ -1531,12 +1531,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>개선 문항에서 "매우 그렇다"고 평가받으면 몇 점이 되나요?</t>
+          <t>동료평가에서 "매우 그렇다"고 답변하면 항상 높은 점수를 받나요?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>개선 문항에서 "매우 그렇다"(5점)로 평가받으면 역산되어 1점이 됩니다. 이는 개선이 필요 없다는 의미로 해석됩니다.</t>
+          <t>아닙니다. 개선 문항(지식3·4, 태도3·4)에서 "매우 그렇다"로 응답하면 역산되어 1점이 됩니다. 예를 들어 "배치 변경을 추천한다"에 "매우 그렇다"고 답하면 불리하게 평가됩니다.</t>
         </is>
       </c>
     </row>
@@ -1548,12 +1548,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>긍정 문항과 개선 문항의 점수 차이는 무엇인가요?</t>
+          <t>동료평가는 어떤 방식으로 진행되나요?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>긍정 문항은 응답 그대로 점수가 적용되고, 개선 문항은 역산됩니다. 예를 들어 개선 문항에서 "그렇지 않다"(2점)고 평가받으면 역산되어 4점이 됩니다.</t>
+          <t>구글폼 기반으로 운영됩니다. 동료를 선택한 후 지식 4문항과 태도 4문항에 5점 척도로 응답하면, 최소 3명 이상이 평가를 제출해야 합니다.</t>
         </is>
       </c>
     </row>
@@ -1565,29 +1565,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>동료평가는 어떤 시스템으로 운영되나요?</t>
+          <t>동료평가 점수 100점 만점에서 70점을 받으면 승진에 영향을 미치나요?</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>구글폼 기반으로 운영됩니다. 동료를 선택한 후 지식과 태도 각 4문항에 응답하는 방식입니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>평가/승진</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>동료평가 문항 중 "이랜드 스피릿을 더 학습하고 실천하면 좋겠습니다"는 어떤 항목인가요?</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>이는 태도 영역의 조직 문화 항목으로, 개선 문항입니다. 조직 문화 적합도를 평가하는 문항이며 역산되어 계산됩니다.</t>
+          <t>70점은 대리 승진의 최소 기준선입니다. 과장 승진을 원한다면 75점 이상, 차장 승진을 원한다면 80점 이상이 필요합니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs 업데이트 (2026-05-29 00:53)
</commit_message>
<xml_diff>
--- a/docs/이랜드건설_동료평가_피어피드백.xlsx
+++ b/docs/이랜드건설_동료평가_피어피드백.xlsx
@@ -1377,7 +1377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1412,12 +1412,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>동료평가(피어피드백)는 몇 년에 몇 번 실시되나요?</t>
+          <t>동료평가(피어피드백)는 몇 년에 한 번 실시되나요?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>연 2회(상반기, 하반기)에 걸쳐 실시됩니다.</t>
+          <t>연 2회 실시됩니다. 상반기와 하반기에 각각 1회씩 진행되며, 구글폼을 통해 운영됩니다.</t>
         </is>
       </c>
     </row>
@@ -1429,12 +1429,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>동료평가에서 최소 몇 명의 평가를 받아야 하나요?</t>
+          <t>동료평가에서 최소 몇 명의 동료로부터 평가를 받아야 하나요?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>최소 3명 이상의 동료로부터 평가를 받아야 합니다.</t>
+          <t>최소 3명 이상의 동료로부터 평가를 받아야 합니다. 동료는 가나다순으로 제시되며, 평가자가 직접 선택합니다.</t>
         </is>
       </c>
     </row>
@@ -1446,12 +1446,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>동료평가 점수는 어떻게 계산되나요?</t>
+          <t>피어피드백 평가 항목은 어떻게 구성되어 있나요?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>지식 4문항과 태도 4문항으로 총 8문항을 5점 척도로 평가합니다. 긍정 문항은 그대로 계산하고, 개선 문항(지식3·4, 태도3·4)은 역산하여 합산한 후 40점 만점을 100점으로 환산합니다.</t>
+          <t>지식(Knowledge) 영역 4문항과 태도(Attitude) 영역 4문항으로 총 8문항으로 구성됩니다. 지식은 직무 전문성, 직무 역량, 성장 필요, 배치 적합성을 평가하고, 태도는 멘토십, 협업·배려, 조직 문화, 대인관계를 평가합니다.</t>
         </is>
       </c>
     </row>
@@ -1463,12 +1463,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>동료평가에서 "개선 문항"이란 무엇인가요?</t>
+          <t>피어피드백 총점이 어떻게 계산되나요?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>개선 문항은 역방향 문항으로, 응답 점수를 역산하여 계산합니다. 지식 3·4번(성장 필요, 배치 적합성)과 태도 3·4번(조직 문화, 대인관계) 4개 문항이 해당됩니다. 예를 들어 "매우 그렇다"에 응답하면 1점으로 역산됩니다.</t>
+          <t>긍정 4문항과 개선(역방향) 4문항의 점수를 모두 합산합니다. 개선 문항은 응답을 역산하여 계산하며, 만점은 40점입니다. 이를 100점 만점으로 환산할 때는 (총점÷40)×100 공식을 적용합니다.</t>
         </is>
       </c>
     </row>
@@ -1480,29 +1480,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>대리로 승진하려면 동료평가 점수가 몇 점 이상이어야 하나요?</t>
+          <t>피어피드백에서 "개선 문항"이란 무엇이고, 왜 점수를 역산하나요?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>대리 승진 시 70점 이상, 과장 승진 시 75점 이상, 차장 승진 시 80점 이상이어야 합니다.</t>
+          <t>개선 문항은 지식3·4, 태도3·4번 항목으로, 직원의 개선 필요 영역을 파악하기 위한 것입니다. 예를 들어 "교육 지원이 필요하다" 또는 "대인관계 교정이 필요하다"에 응답합니다. 점수는 역산되므로, "매우 그렇다(5점)"라고 답하면 1점으로 계산되어 개선이 불필요함을 의미합니다.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>평가/승진</t>
+          <t>평evaluation/승진</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>동료평가의 지식 영역에서는 어떤 항목들을 평가하나요?</t>
+          <t>대리로 승진하려면 피어피드백 점수가 얼마 이상이어야 하나요?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>직무 전문성(사내 강사 추천 여부), 직무 역량(연차 대비 역량 수준), 성장 필요도, 배치 적합성 등 4개 항목을 평가합니다.</t>
+          <t>대리 승진 시 피어피드백 점수 70점 이상이 필요합니다. 과장 승진은 75점 이상, 차장 승진은 80점 이상의 점수가 요구됩니다.</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>동료평가의 태도 영역에서는 어떤 항목들을 평가하나요?</t>
+          <t>피어피드백에서 "매우 그렇다"라고 받은 평가는 항상 좋은 평가인가요?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>멘토십(인격적 멘토 역할), 협업·배려(동료 배려 및 존중), 조직 문화(이랜드 스피릿 실천), 대인관계(관계 개선 필요도) 등 4개 항목을 평가합니다.</t>
+          <t>아니요, 긍정 문항(지식1·2, 태도1·2)에서는 "매우 그렇다"가 5점으로 높은 평가이지만, 개선 문항(지식3·4, 태도3·4)에서는 역산되어 1점이 됩니다. 개선 문항에서는 "전혀 아니다"가 5점으로 가장 좋은 평가입니다.</t>
         </is>
       </c>
     </row>
@@ -1531,12 +1531,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>동료평가에서 "매우 그렇다"고 답변하면 항상 높은 점수를 받나요?</t>
+          <t>내가 받은 피어피드백 평가 결과는 어떻게 확인하나요?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>아닙니다. 개선 문항(지식3·4, 태도3·4)에서 "매우 그렇다"로 응답하면 역산되어 1점이 됩니다. 예를 들어 "배치 변경을 추천한다"에 "매우 그렇다"고 답하면 불리하게 평가됩니다.</t>
+          <t>HR팀이 수집한 데이터를 엑셀로 다운로드하여 분석합니다. 결과 공지 일정은 별도로 안내되며, 개별 피드백은 인사팀을 통해 확인할 수 있습니다.</t>
         </is>
       </c>
     </row>
@@ -1548,12 +1548,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>동료평가는 어떤 방식으로 진행되나요?</t>
+          <t>"인격적인 멘토 역할을 해줄 수 있는 직원"이라는 평가 항목은 무엇을 의미하나요?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>구글폼 기반으로 운영됩니다. 동료를 선택한 후 지식 4문항과 태도 4문항에 5점 척도로 응답하면, 최소 3명 이상이 평가를 제출해야 합니다.</t>
+          <t>이는 태도 1번 항목으로, 해당 직원이 리더십과 후배 육성 능력을 갖추었는지 평가하는 것입니다. 인격적이고 신뢰할 수 있는 멘토 역할을 할 수 있는 역량이 있는지를 동료들이 평가합니다.</t>
         </is>
       </c>
     </row>
@@ -1565,12 +1565,63 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>동료평가 점수 100점 만점에서 70점을 받으면 승진에 영향을 미치나요?</t>
+          <t>"이랜드 스피릿을 더 학습하고 실천하면 좋겠다"는 평가를 받으면 어떻게 해석해야 하나요?</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>70점은 대리 승진의 최소 기준선입니다. 과장 승진을 원한다면 75점 이상, 차장 승진을 원한다면 80점 이상이 필요합니다.</t>
+          <t>이는 태도 3번 항목으로, 조직 문화 적합도를 평가하는 개선 문항입니다. 이 항목에서 높은 점수를 받으면 회사의 이랜드 스피릿을 더 잘 학습하고 실천할 필요가 있다는 의미입니다. 점수는 역산되므로 낮은 응답이 높은 평가가 됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>평가/승진</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>"함께하는 직원들을 배려하고 존중한다"는 평가는 무엇을 평가하는 항목인가요?</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>이는 태도 2번 항목으로, 협업·배려 능력과 팀 내 관계 및 소통 능력을 평가합니다. 동료들과의 관계에서 배려심과 존중하는 태도가 있는지를 평가하는 것입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>평가/승진</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>지식 4번 "직무 변경 또는 부서 재배치를 추천합니다"는 항목에서 높은 점수가 나오면 어떤 의미인가요?</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>이는 개선 문항으로 역산되므로, 높은 응답은 낮은 점수가 됩니다. 만약 "매우 그렇다"라고 평가받으면 1점이 되어, 현재 직무가 맞지 않으므로 변경이 필요하다는 의미입니다. 이 경우 인사팀과 상담하여 직무 적합성을 재검토할 수 있습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>평가/승진</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>피어피드백에서 연차에 맞는 역량이 있는지 평가하는 항목은 어떤 것인가요?</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>지식 2번 항목 "연차에 맞는 직무 역량을 가지고 있습니다"가 이를 평가합니다. 이는 긍정 문항으로, 현재 근무 연차에 적합한 수준의 직무 역량을 갖추었는지를 동료들이 평가합니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs 업데이트 (2026-05-29 01:04)
</commit_message>
<xml_diff>
--- a/docs/이랜드건설_동료평가_피어피드백.xlsx
+++ b/docs/이랜드건설_동료평가_피어피드백.xlsx
@@ -1176,6 +1176,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
@@ -1376,7 +1377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1411,12 +1412,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>동료평가(피어피드백)는 몇 년에 한 번 실시되나요?</t>
+          <t>동료평가(피어피드백)는 연 몇 회 실시되나요?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>연 2회 실시됩니다. 상반기와 하반기에 각각 1회씩 진행되며, 구글폼을 통해 운영됩니다.</t>
+          <t>연 2회(상반기, 하반기) 실시됩니다.</t>
         </is>
       </c>
     </row>
@@ -1428,12 +1429,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>동료평가에서 최소 몇 명의 동료로부터 평가를 받아야 하나요?</t>
+          <t>동료평가에서 최소 몇 명 이상의 평가를 받아야 하나요?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>최소 3명 이상의 동료로부터 평가를 받아야 합니다. 동료는 가나다순으로 제시되며, 평가자가 직접 선택합니다.</t>
+          <t>최소 3명 이상의 동료로부터 평가를 받아야 합니다.</t>
         </is>
       </c>
     </row>
@@ -1445,12 +1446,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>피어피드백 평가 항목은 어떻게 구성되어 있나요?</t>
+          <t>동료평가 문항은 어떻게 구성되어 있나요?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>지식(Knowledge) 영역 4문항과 태도(Attitude) 영역 4문항으로 총 8문항으로 구성됩니다. 지식은 직무 전문성, 직무 역량, 성장 필요, 배치 적합성을 평가하고, 태도는 멘토십, 협업·배려, 조직 문화, 대인관계를 평가합니다.</t>
+          <t>지식 영역 4문항(직무 전문성, 직무 역량, 성장 필요, 배치 적합성)과 태도 영역 4문항(멘토십, 협업·배려, 조직문화, 대인관계)으로 총 8문항으로 구성됩니다.</t>
         </is>
       </c>
     </row>
@@ -1462,12 +1463,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>피어피드백 총점이 어떻게 계산되나요?</t>
+          <t>동료평가 점수는 어떻게 계산되나요?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>긍정 4문항과 개선(역방향) 4문항의 점수를 모두 합산합니다. 개선 문항은 응답을 역산하여 계산하며, 만점은 40점입니다. 이를 100점 만점으로 환산할 때는 (총점÷40)×100 공식을 적용합니다.</t>
+          <t>긍정 4문항의 점수를 합산하고 개선 4문항은 역산하여 합산한 후, 총점을 40으로 나누어 100점으로 환산합니다. (총점/40×100)</t>
         </is>
       </c>
     </row>
@@ -1479,12 +1480,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>피어피드백에서 "개선 문항"이란 무엇이고, 왜 점수를 역산하나요?</t>
+          <t>대리로 승진하려면 피어피드백 점수가 몇 점 이상이어야 하나요?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>개선 문항은 지식3·4, 태도3·4번 항목으로, 직원의 개선 필요 영역을 파악하기 위한 것입니다. 예를 들어 "교육 지원이 필요하다" 또는 "대인관계 교정이 필요하다"에 응답합니다. 점수는 역산되므로, "매우 그렇다(5점)"라고 답하면 1점으로 계산되어 개선이 불필요함을 의미합니다.</t>
+          <t>대리 승진 시 피어피드백 70점 이상이 필요합니다.</t>
         </is>
       </c>
     </row>
@@ -1496,12 +1497,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>대리로 승진하려면 피어피드백 점수가 얼마 이상이어야 하나요?</t>
+          <t>과장으로 승진하려면 피어피드백 점수가 몇 점 이상이어야 하나요?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>대리 승진 시 피어피드백 점수 70점 이상이 필요합니다. 과장 승진은 75점 이상, 차장 승진은 80점 이상의 점수가 요구됩니다.</t>
+          <t>과장 승진 시 피어피드백 75점 이상이 필요합니다.</t>
         </is>
       </c>
     </row>
@@ -1513,12 +1514,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>피어피드백에서 "매우 그렇다"라고 받은 평가는 항상 좋은 평가인가요?</t>
+          <t>차장으로 승진하려면 피어피드백 점수가 몇 점 이상이어야 하나요?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>아니요, 긍정 문항(지식1·2, 태도1·2)에서는 "매우 그렇다"가 5점으로 높은 평가이지만, 개선 문항(지식3·4, 태도3·4)에서는 역산되어 1점이 됩니다. 개선 문항에서는 "전혀 아니다"가 5점으로 가장 좋은 평가입니다.</t>
+          <t>차장 승진 시 피어피드백 80점 이상이 필요합니다.</t>
         </is>
       </c>
     </row>
@@ -1530,12 +1531,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>내가 받은 피어피드백 평가 결과는 어떻게 확인하나요?</t>
+          <t>"성장 필요" 문항에서 높은 점수를 받으면 어떻게 되나요?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>HR팀이 수집한 데이터를 엑셀로 다운로드하여 분석합니다. 결과 공지 일정은 별도로 안내되며, 개별 피드백은 인사팀을 통해 확인할 수 있습니다.</t>
+          <t>"성장 필요"는 개선 문항으로 역산되기 때문에 높은 점수(매우 그렇다)를 받으면 역산되어 1점이 되어 전체 점수가 낮아집니다.</t>
         </is>
       </c>
     </row>
@@ -1547,12 +1548,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>"인격적인 멘토 역할을 해줄 수 있는 직원"이라는 평가 항목은 무엇을 의미하나요?</t>
+          <t>"배치 적합성" 문항에서 "직무 변경을 추천한다"는 높은 평가를 받으면 어떻게 되나요?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>이는 태도 1번 항목으로, 해당 직원이 리더십과 후배 육성 능력을 갖추었는지 평가하는 것입니다. 인격적이고 신뢰할 수 있는 멘토 역할을 할 수 있는 역량이 있는지를 동료들이 평가합니다.</t>
+          <t>"배치 적합성"도 개선 문항으로 역산되므로, 높은 평가를 받으면 역산되어 낮은 점수가 되어 전체 평가점수에 불리하게 작용합니다.</t>
         </is>
       </c>
     </row>
@@ -1564,12 +1565,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>"이랜드 스피릿을 더 학습하고 실천하면 좋겠다"는 평가를 받으면 어떻게 해석해야 하나요?</t>
+          <t>동료평가에서 5점 척도는 어떻게 구성되어 있나요?</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>이는 태도 3번 항목으로, 조직 문화 적합도를 평가하는 개선 문항입니다. 이 항목에서 높은 점수를 받으면 회사의 이랜드 스피릿을 더 잘 학습하고 실천할 필요가 있다는 의미입니다. 점수는 역산되므로 낮은 응답이 높은 평가가 됩니다.</t>
+          <t>매우 그렇다(5), 그렇다(4), 보통이다(3), 그렇지 않다(2), 전혀 아니다(1)의 5단계 척도입니다.</t>
         </is>
       </c>
     </row>
@@ -1581,12 +1582,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>"함께하는 직원들을 배려하고 존중한다"는 평가는 무엇을 평가하는 항목인가요?</t>
+          <t>동료평가는 어떤 방식으로 진행되나요?</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>이는 태도 2번 항목으로, 협업·배려 능력과 팀 내 관계 및 소통 능력을 평가합니다. 동료들과의 관계에서 배려심과 존중하는 태도가 있는지를 평가하는 것입니다.</t>
+          <t>구글폼을 기반으로 운영되며, 동료를 선택한 후 지식/태도 각 4문항에 응답하는 방식입니다.</t>
         </is>
       </c>
     </row>
@@ -1598,29 +1599,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>지식 4번 "직무 변경 또는 부서 재배치를 추천합니다"는 항목에서 높은 점수가 나오면 어떤 의미인가요?</t>
+          <t>개선 문항(역방향 문항)에서 "전혀 아니다"라고 평가받으면 어떻게 되나요?</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>이는 개선 문항으로 역산되므로, 높은 응답은 낮은 점수가 됩니다. 만약 "매우 그렇다"라고 평가받으면 1점이 되어, 현재 직무가 맞지 않으므로 변경이 필요하다는 의미입니다. 이 경우 인사팀과 상담하여 직무 적합성을 재검토할 수 있습니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>평가/승진</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>피어피드백에서 연차에 맞는 역량이 있는지 평가하는 항목은 어떤 것인가요?</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>지식 2번 항목 "연차에 맞는 직무 역량을 가지고 있습니다"가 이를 평가합니다. 이는 긍정 문항으로, 현재 근무 연차에 적합한 수준의 직무 역량을 갖추었는지를 동료들이 평가합니다.</t>
+          <t>역산되어 5점이 되어 전체 점수에 긍정적으로 작용합니다. 예를 들어 성장 필요나 배치 변경이 "전혀 아니다"는 것은 직원이 잘하고 있다는 의미입니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs 업데이트 (2026-05-29 01:06)
</commit_message>
<xml_diff>
--- a/docs/이랜드건설_동료평가_피어피드백.xlsx
+++ b/docs/이랜드건설_동료평가_피어피드백.xlsx
@@ -1377,7 +1377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1412,12 +1412,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>동료평가(피어피드백)는 연 몇 회 실시되나요?</t>
+          <t>동료평가(피어피드백)는 연간 몇 회 실시되나요?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>연 2회(상반기, 하반기) 실시됩니다.</t>
+          <t>연 2회(상반기, 하반기)에 걸쳐 실시됩니다.</t>
         </is>
       </c>
     </row>
@@ -1446,12 +1446,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>동료평가 문항은 어떻게 구성되어 있나요?</t>
+          <t>동료평가(피어피드백)의 평가 문항은 몇 개인가요?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>지식 영역 4문항(직무 전문성, 직무 역량, 성장 필요, 배치 적합성)과 태도 영역 4문항(멘토십, 협업·배려, 조직문화, 대인관계)으로 총 8문항으로 구성됩니다.</t>
+          <t>지식 4문항, 태도 4문항으로 총 8문항입니다.</t>
         </is>
       </c>
     </row>
@@ -1463,12 +1463,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>동료평가 점수는 어떻게 계산되나요?</t>
+          <t>동료평가에서 '개선 문항'이란 무엇인가요?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>긍정 4문항의 점수를 합산하고 개선 4문항은 역산하여 합산한 후, 총점을 40으로 나누어 100점으로 환산합니다. (총점/40×100)</t>
+          <t>개선 문항은 역방향으로 설계되어 점수가 역산되는 문항입니다. 예를 들어 '교육 지원이 필요하다'에 "매우 그렇다"고 답하면 1점으로 역산되어, 역량 부족을 의미합니다.</t>
         </is>
       </c>
     </row>
@@ -1480,12 +1480,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>대리로 승진하려면 피어피드백 점수가 몇 점 이상이어야 하나요?</t>
+          <t>동료평가의 만점은 몇 점이고, 100점으로 어떻게 환산되나요?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>대리 승진 시 피어피드백 70점 이상이 필요합니다.</t>
+          <t>만점은 40점이며, 100점 환산 공식은 (총점÷40)×100입니다. 예를 들어 32점을 받으면 80점으로 환산됩니다.</t>
         </is>
       </c>
     </row>
@@ -1497,12 +1497,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>과장으로 승진하려면 피어피드백 점수가 몇 점 이상이어야 하나요?</t>
+          <t>대리로 승진하려면 동료평가에서 최소 몇 점을 받아야 하나요?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>과장 승진 시 피어피드백 75점 이상이 필요합니다.</t>
+          <t>70점 이상을 받아야 합니다.</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>차장으로 승진하려면 피어피드백 점수가 몇 점 이상이어야 하나요?</t>
+          <t>과장으로 승진하려면 동료평가에서 최소 몇 점을 받아야 하나요?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>차장 승진 시 피어피드백 80점 이상이 필요합니다.</t>
+          <t>75점 이상을 받아야 합니다.</t>
         </is>
       </c>
     </row>
@@ -1531,12 +1531,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>"성장 필요" 문항에서 높은 점수를 받으면 어떻게 되나요?</t>
+          <t>차장으로 승진하려면 동료평가에서 최소 몇 점을 받아야 하나요?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>"성장 필요"는 개선 문항으로 역산되기 때문에 높은 점수(매우 그렇다)를 받으면 역산되어 1점이 되어 전체 점수가 낮아집니다.</t>
+          <t>80점 이상을 받아야 합니다.</t>
         </is>
       </c>
     </row>
@@ -1548,12 +1548,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>"배치 적합성" 문항에서 "직무 변경을 추천한다"는 높은 평가를 받으면 어떻게 되나요?</t>
+          <t>동료평가에서 "인격적인 멘토 역할"은 어떤 능력을 평가하는 항목인가요?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>"배치 적합성"도 개선 문항으로 역산되므로, 높은 평가를 받으면 역산되어 낮은 점수가 되어 전체 평가점수에 불리하게 작용합니다.</t>
+          <t>리더십과 후배 육성 능력을 평가하는 멘토십 항목입니다.</t>
         </is>
       </c>
     </row>
@@ -1565,12 +1565,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>동료평가에서 5점 척도는 어떻게 구성되어 있나요?</t>
+          <t>동료평가에서 "함께하는 직원들을 배려하고 존중"한다는 항목은 무엇을 평가하나요?</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>매우 그렇다(5), 그렇다(4), 보통이다(3), 그렇지 않다(2), 전혀 아니다(1)의 5단계 척도입니다.</t>
+          <t>팀 내 관계 및 소통 능력을 평가하는 협업·배려 항목입니다.</t>
         </is>
       </c>
     </row>
@@ -1582,12 +1582,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>동료평가는 어떤 방식으로 진행되나요?</t>
+          <t>동료평가를 받을 때 누가 나를 평가하나요?</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>구글폼을 기반으로 운영되며, 동료를 선택한 후 지식/태도 각 4문항에 응답하는 방식입니다.</t>
+          <t>구글폼을 통해 동료들이 가나다순으로 선택된 후 평가합니다.</t>
         </is>
       </c>
     </row>
@@ -1599,12 +1599,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>개선 문항(역방향 문항)에서 "전혀 아니다"라고 평가받으면 어떻게 되나요?</t>
+          <t>동료평가의 5점 척도는 무엇인가요?</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>역산되어 5점이 되어 전체 점수에 긍정적으로 작용합니다. 예를 들어 성장 필요나 배치 변경이 "전혀 아니다"는 것은 직원이 잘하고 있다는 의미입니다.</t>
+          <t>"매우 그렇다(5점), 그렇다(4점), 보통이다(3점), 그렇지 않다(2점), 전혀 아니다(1점)"로 구성됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>평가/승진</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>"이랜드 스피릿을 더 학습하고 실천하면 좋겠다"는 항목은 무엇을 평가하나요?</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>조직 문화 적합도를 평가하는 항목으로, 회사의 가치관과 문화에 얼마나 부합하는지를 평가합니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs 업데이트 (2026-05-29 01:27)
</commit_message>
<xml_diff>
--- a/docs/이랜드건설_동료평가_피어피드백.xlsx
+++ b/docs/이랜드건설_동료평가_피어피드백.xlsx
@@ -1377,7 +1377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1412,12 +1412,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>동료평가(피어피드백)는 연간 몇 회 실시되나요?</t>
+          <t>동료평가(피어피드백)는 연 몇 회 실시되나요?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>연 2회(상반기, 하반기)에 걸쳐 실시됩니다.</t>
+          <t>연 2회(상반기, 하반기) 실시됩니다.</t>
         </is>
       </c>
     </row>
@@ -1446,12 +1446,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>동료평가(피어피드백)의 평가 문항은 몇 개인가요?</t>
+          <t>동료평가 문항은 어떻게 구성되어 있나요?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>지식 4문항, 태도 4문항으로 총 8문항입니다.</t>
+          <t>지식 영역 4문항(직무 전문성, 직무 역량, 성장 필요, 배치 적합성)과 태도 영역 4문항(멘토십, 협업·배려, 조직 문화, 대인관계)으로 총 8개 문항으로 구성되어 있습니다.</t>
         </is>
       </c>
     </row>
@@ -1463,12 +1463,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>동료평가에서 '개선 문항'이란 무엇인가요?</t>
+          <t>동료평가는 어떤 방식으로 진행되나요?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>개선 문항은 역방향으로 설계되어 점수가 역산되는 문항입니다. 예를 들어 '교육 지원이 필요하다'에 "매우 그렇다"고 답하면 1점으로 역산되어, 역량 부족을 의미합니다.</t>
+          <t>구글폼을 통해 동료를 선택(가나다순)한 후 지식/태도 각 4문항을 5점 척도로 응답하는 방식으로 진행됩니다.</t>
         </is>
       </c>
     </row>
@@ -1480,12 +1480,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>동료평가의 만점은 몇 점이고, 100점으로 어떻게 환산되나요?</t>
+          <t>동료평가 총점은 어떻게 산정되나요?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>만점은 40점이며, 100점 환산 공식은 (총점÷40)×100입니다. 예를 들어 32점을 받으면 80점으로 환산됩니다.</t>
+          <t>긍정 4문항의 합산점수와 개선 문항 4개의 역산 합산점수를 더한 후, 총점을 40으로 나누어 100점으로 환산합니다.</t>
         </is>
       </c>
     </row>
@@ -1497,12 +1497,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>대리로 승진하려면 동료평가에서 최소 몇 점을 받아야 하나요?</t>
+          <t>승진 시 필요한 동료평가 점수는 얼마나 되나요?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>70점 이상을 받아야 합니다.</t>
+          <t>대리 승진 시 70점 이상, 과장 승진 시 75점 이상, 차장 승진 시 80점 이상이 필요합니다.</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>과장으로 승진하려면 동료평가에서 최소 몇 점을 받아야 하나요?</t>
+          <t>개선 문항에서 "매우 그렇다"고 평가받으면 어떻게 되나요?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>75점 이상을 받아야 합니다.</t>
+          <t>개선 문항은 역산되므로 "매우 그렇다"(5점)는 1점으로 처리되어 개선이 필요 없는 것으로 해석됩니다.</t>
         </is>
       </c>
     </row>
@@ -1531,12 +1531,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>차장으로 승진하려면 동료평가에서 최소 몇 점을 받아야 하나요?</t>
+          <t>"보통이다"로 평가받은 경우 점수는 어떻게 되나요?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>80점 이상을 받아야 합니다.</t>
+          <t>긍정 문항과 개선 문항 모두 "보통이다"(3점)는 3점으로 동일하게 처리됩니다.</t>
         </is>
       </c>
     </row>
@@ -1548,12 +1548,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>동료평가에서 "인격적인 멘토 역할"은 어떤 능력을 평가하는 항목인가요?</t>
+          <t>동료평가에서 직무 변경이나 부서 재배치를 추천받으면 어떤 영향이 있나요?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>리더십과 후배 육성 능력을 평가하는 멘토십 항목입니다.</t>
+          <t>"직무 변경 또는 부서 재배치를 추천합니다"는 개선 문항으로, 높은 점수를 받으면 역산되어 총점에 부정적으로 반영될 수 있습니다.</t>
         </is>
       </c>
     </row>
@@ -1565,63 +1565,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>동료평가에서 "함께하는 직원들을 배려하고 존중"한다는 항목은 무엇을 평가하나요?</t>
+          <t>조직 문화 적합도는 어떻게 평가되나요?</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>팀 내 관계 및 소통 능력을 평가하는 협업·배려 항목입니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>평가/승진</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>동료평가를 받을 때 누가 나를 평가하나요?</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>구글폼을 통해 동료들이 가나다순으로 선택된 후 평가합니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>평가/승진</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>동료평가의 5점 척도는 무엇인가요?</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>"매우 그렇다(5점), 그렇다(4점), 보통이다(3점), 그렇지 않다(2점), 전혀 아니다(1점)"로 구성됩니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>평가/승진</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>"이랜드 스피릿을 더 학습하고 실천하면 좋겠다"는 항목은 무엇을 평가하나요?</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>조직 문화 적합도를 평가하는 항목으로, 회사의 가치관과 문화에 얼마나 부합하는지를 평가합니다.</t>
+          <t>"이랜드 스피릿을 더 학습하고 실천하면 좋겠습니다"라는 개선 문항으로 평가되며, 역산되어 조직문화 적합도가 반영됩니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs 업데이트 (2026-05-29 20:05)
</commit_message>
<xml_diff>
--- a/docs/이랜드건설_동료평가_피어피드백.xlsx
+++ b/docs/이랜드건설_동료평가_피어피드백.xlsx
@@ -1377,7 +1377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1412,12 +1412,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>동료평가(피어피드백)는 몇 명이 평가해야 하나요?</t>
+          <t>동료평가(피어피드백)는 몇 명에게 받아야 하나요?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>최소 3명 이상의 동료로부터 평가를 받아야 합니다. 구글폼을 통해 동료를 선택한 후 지식과 태도 영역의 문항에 응답하게 됩니다.</t>
+          <t>최소 3명 이상으로부터 평가를 받아야 합니다. 구글폼을 통해 동료를 선택한 후 지식 4문항, 태도 4문항에 응답하는 방식으로 진행됩니다.</t>
         </is>
       </c>
     </row>
@@ -1429,12 +1429,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>동료평가는 연간 몇 회 실시되나요?</t>
+          <t>동료평가는 몇 번 실시되나요?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>연 2회 실시됩니다. 상반기와 하반기에 각각 1회씩 진행됩니다.</t>
+          <t>연 2회(상반기, 하반기)로 실시됩니다.</t>
         </is>
       </c>
     </row>
@@ -1446,12 +1446,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>동료평가의 평가 영역은 어떻게 구성되어 있나요?</t>
+          <t>동료평가 지식(Knowledge) 영역에서는 어떤 항목들을 평가하나요?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>지식(Knowledge) 영역 4문항과 태도(Attitude) 영역 4문항으로 총 8문항으로 구성됩니다. 지식 영역은 직무 전문성, 직무 역량, 성장 필요, 배치 적합성을 평가하며, 태도 영역은 멘토십, 협업·배려, 조직 문화, 대인관계를 평가합니다.</t>
+          <t>직무 전문성, 직무 역량, 성장 필요성, 배치 적합성 총 4개 문항으로 구성되어 있습니다. 구체적으로는 사내 강사 추천 여부, 연차 대비 역량 수준, 교육 지원 필요 여부, 부서 재배치 필요 여부를 평가합니다.</t>
         </is>
       </c>
     </row>
@@ -1463,12 +1463,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>동료평가 점수는 어떻게 산정되나요?</t>
+          <t>동료평가 태도(Attitude) 영역에서는 어떤 항목들을 평가하나요?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>총 8문항 중 긍정 문항 4개와 개선(역방향) 문항 4개로 나뉩니다. 긍정 문항은 응답 그대로 점수(5~1점)가 반영되며, 개선 문항은 역산되어 반영됩니다(매우 그렇다=1점, 그렇지 않다=4점, 전혀 아니다=5점). 모든 점수를 합산하면 만점 40점이 되며, 이를 100점으로 환산합니다. (총점÷40×100)</t>
+          <t>멘토십, 협업·배려, 조직 문화, 대인관계 총 4개 문항으로 구성되어 있습니다. 구체적으로는 멘토 역할 적합성, 배려와 존중, 이랜드 스피릿 실천 수준, 대인관계 상태를 평가합니다.</t>
         </is>
       </c>
     </row>
@@ -1480,12 +1480,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>대리 승진을 위한 동료평가 최소 점수는 몇 점인가요?</t>
+          <t>동료평가에서 '개선 문항'이란 무엇인가요?</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>70점 이상이어야 합니다.</t>
+          <t>지식 3·4번 문항과 태도 3·4번 문항으로, 응답 점수를 역산하여 계산합니다. 예를 들어 '같은 연차 직원들에 비해 교육 지원이 필요하다'는 질문에 '매우 그렇다'고 답하면 1점(역산)이 되어 개선이 필요 없는 것으로 해석됩니다.</t>
         </is>
       </c>
     </row>
@@ -1497,12 +1497,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>과장 승진을 위한 동료평가 최소 점수는 몇 점인가요?</t>
+          <t>동료평가 점수는 어떻게 계산되나요?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>75점 이상이어야 합니다.</t>
+          <t>긍정 4문항 점수를 합산한 후, 개선 4문항을 역산한 점수를 더합니다. 총점은 만점 40점이며, 이를 100점 만점으로 환산합니다. (총점÷40×100)</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>차장 승진을 위한 동료평가 최소 점수는 몇 점인가요?</t>
+          <t>대리로 승진하려면 동료평가 점수가 어느 정도 필요한가요?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>80점 이상이어야 합니다.</t>
+          <t>70점 이상이어야 합니다.</t>
         </is>
       </c>
     </row>
@@ -1531,12 +1531,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>"개선 문항"에서 "매우 그렇다"고 응답하면 어떻게 되나요?</t>
+          <t>과장으로 승진하려면 동료평가 점수가 어느 정도 필요한가요?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>역산되어 1점만 반영됩니다. 예를 들어 "직무 변경 또는 부서 재배치를 추천합니다"에 "매우 그렇다"고 응답하면 개선이 필요하지 않다는 의미로 해석되어 불이익을 받을 수 있습니다.</t>
+          <t>75점 이상이어야 합니다.</t>
         </is>
       </c>
     </row>
@@ -1548,12 +1548,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>"개선 문항"에서 "전혀 아니다"고 응답하면 어떻게 되나요?</t>
+          <t>차장으로 승진하려면 동료평가 점수가 어느 정도 필요한가요?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>역산되어 5점이 반영됩니다. 이는 개선이 필요 없다는 긍정적인 의미로 해석되어 높은 점수를 받습니다.</t>
+          <t>80점 이상이어야 합니다.</t>
         </is>
       </c>
     </row>
@@ -1565,12 +1565,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>동료평가에서 "직무 전문성"을 평가하는 문항은 무엇인가요?</t>
+          <t>동료평가에서 5점 척도는 어떻게 되나요?</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>"해당 직무의 사내 강사로 추천하고 싶습니다"라는 문항으로, 직무 전문성의 최상위 수준을 평가합니다.</t>
+          <t>'매우 그렇다(5점)', '그렇다(4점)', '보통이다(3점)', '그렇지 않다(2점)', '전혀 아니다(1점)'로 구성됩니다.</t>
         </is>
       </c>
     </row>
@@ -1582,63 +1582,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>연차에 맞는 역량 수준을 평가하는 문항은 무엇인가요?</t>
+          <t>동료평가 점수가 낮으면 어떤 영향이 있나요?</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>"연차에 맞는 직무 역량을 가지고 있습니다"라는 문항으로, 같은 연차의 다른 직원과 비교하여 역량 수준을 평가합니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>평가/승진</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>리더십과 후배 육성 능력은 어떤 문항으로 평가되나요?</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>"인격적인 멘토 역할을 해줄 수 있는 직원입니다"라는 태도 영역의 문항으로 평가됩니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>평가/승진</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>팀 내 협업과 관계 능력을 평가하는 문항은 무엇인가요?</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>"함께하는 직원들을 배려하고 존중합니다"라는 문항으로, 팀 내 관계와 소통 능력을 평가합니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>평가/승진</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>조직 문화 적응도를 평가하는 문항은 무엇인가요?</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>"이랜드 스피릿을 더 학습하고 실천하면 좋겠습니다"라는 문항으로, 역방향 문항으로 평가되어 조직문화에 대한 적합도를 측정합니다.</t>
+          <t>승진 시 필요한 최소 점수에 미달하면 승진이 불가능합니다. 또한 개선이 필요한 영역에서 낮은 점수를 받으면 향후 교육·코칭 등의 인사관리 대상이 될 수 있습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>